<commit_message>
use TMP directory instead of outputs
</commit_message>
<xml_diff>
--- a/outputs/reanalysis2/zones/mites.xlsx
+++ b/outputs/reanalysis2/zones/mites.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="stones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="town" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="dead" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="alive" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -159,7 +159,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6667500" cy="3810000"/>
+    <ext cx="6667500" cy="32385000"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -184,7 +184,7 @@
       <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2952750" cy="533400"/>
+    <ext cx="3105150" cy="1066800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -192,6 +192,56 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>18</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3086100" cy="1028700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>18</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2952750" cy="1028700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -214,7 +264,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6667500" cy="5715000"/>
+    <ext cx="6667500" cy="22860000"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -239,7 +289,7 @@
       <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="3095625" cy="533400"/>
+    <ext cx="3105150" cy="1028700"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -247,6 +297,56 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>18</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2914650" cy="1028700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>18</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2924175" cy="990600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -549,7 +649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:U35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -591,7 +691,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>mite_0070</t>
+          <t>mite_0000</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -609,9 +709,9 @@
           <t>dead</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>alive</t>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -638,22 +738,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>mite_0081</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>alive</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>alive</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>alive</t>
+          <t>mite_0001</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -661,9 +761,9 @@
           <t>dead</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>alive</t>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -685,17 +785,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>mite_0108</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>alive</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>alive</t>
+          <t>mite_0002</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -718,12 +818,1469 @@
           <t>dead</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>alive</t>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>mite_0004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>mite_0005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>mite_0007</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>mite_0008</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>mite_0009</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>mite_0010</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>mite_0011</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>mite_0013</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>mite_0014</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>mite_0016</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>mite_0018</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>mite_0020</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>mite_0022</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>mite_0028</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>mite_0030</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>mite_0031</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>mite_0032</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>mite_0035</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>mite_0036</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>mite_0037</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>mite_0039</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>mite_0040</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>mite_0041</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>mite_0042</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>mite_0045</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>mite_0047</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>mite_0051</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>mite_0054</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>mite_0055</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>mite_0056</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>mite_0057</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>dead</t>
         </is>
@@ -744,7 +2301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U6"/>
+  <dimension ref="A1:U24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -786,7 +2343,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>mite_0082</t>
+          <t>mite_0003</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -804,19 +2361,19 @@
           <t>alive</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>dead</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>dead</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>alive</t>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -824,16 +2381,16 @@
           <t>dead</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>alive</t>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>mite_0085</t>
+          <t>mite_0006</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -846,24 +2403,24 @@
           <t>alive</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>dead</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>dead</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>dead</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>dead</t>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -871,26 +2428,26 @@
           <t>alive</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>dead</t>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>mite_0091</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>alive</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>alive</t>
+          <t>mite_0012</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -898,9 +2455,9 @@
           <t>dead</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>dead</t>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -908,14 +2465,14 @@
           <t>dead</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>alive</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>alive</t>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -927,17 +2484,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>mite_0106</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>dead</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>dead</t>
+          <t>mite_0017</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -945,46 +2502,46 @@
           <t>dead</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>dead</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>dead</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>dead</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>dead</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>dead</t>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>mite_0107</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>alive</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>dead</t>
+          <t>mite_0019</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -992,9 +2549,9 @@
           <t>dead</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>dead</t>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1002,9 +2559,9 @@
           <t>dead</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>dead</t>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1013,6 +2570,852 @@
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>mite_0021</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>mite_0023</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>mite_0024</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>mite_0025</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>mite_0026</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>mite_0027</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>mite_0029</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>mite_0033</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>mite_0034</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>mite_0038</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>mite_0043</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>mite_0044</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>mite_0046</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>mite_0048</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>mite_0049</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>mite_0050</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>mite_0052</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>mite_0053</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>dead</t>
         </is>

</xml_diff>